<commit_message>
Auto-conversión de datos meteorológicos a CSV y XLSX
</commit_message>
<xml_diff>
--- a/downld02.xlsx
+++ b/downld02.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH75"/>
+  <dimension ref="A1:AH77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -9768,6 +9768,258 @@
         <v>30</v>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>10/09/26</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="D76" s="4" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="E76" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="F76" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="G76" s="4" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="H76" s="4" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="I76" s="3" t="inlineStr">
+        <is>
+          <t>NNE</t>
+        </is>
+      </c>
+      <c r="J76" s="4" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="K76" s="4" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="L76" s="3" t="inlineStr">
+        <is>
+          <t>NNE</t>
+        </is>
+      </c>
+      <c r="M76" s="4" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="N76" s="4" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="O76" s="4" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="P76" s="3" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="Q76" s="4" t="n">
+        <v>1006.3</v>
+      </c>
+      <c r="R76" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S76" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T76" s="3" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="U76" s="3" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="V76" s="3" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="W76" s="3" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="X76" s="3" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="Y76" s="3" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="Z76" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA76" s="4" t="n">
+        <v>0.184</v>
+      </c>
+      <c r="AB76" s="4" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="AC76" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="AD76" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE76" s="5" t="n">
+        <v>640</v>
+      </c>
+      <c r="AF76" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="AG76" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="AH76" s="5" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t>10/09/26</t>
+        </is>
+      </c>
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="D77" s="7" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="E77" s="7" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="F77" s="8" t="n">
+        <v>48</v>
+      </c>
+      <c r="G77" s="7" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="H77" s="7" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="I77" s="6" t="inlineStr">
+        <is>
+          <t>SE</t>
+        </is>
+      </c>
+      <c r="J77" s="7" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="K77" s="7" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="L77" s="6" t="inlineStr">
+        <is>
+          <t>ENE</t>
+        </is>
+      </c>
+      <c r="M77" s="7" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="N77" s="7" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="O77" s="7" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="P77" s="6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="Q77" s="7" t="n">
+        <v>1005.2</v>
+      </c>
+      <c r="R77" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S77" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T77" s="6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="U77" s="6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="V77" s="6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="W77" s="6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="X77" s="6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="Y77" s="6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="Z77" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA77" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AB77" s="7" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="AC77" s="8" t="n">
+        <v>57</v>
+      </c>
+      <c r="AD77" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE77" s="8" t="n">
+        <v>640</v>
+      </c>
+      <c r="AF77" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="AG77" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="AH77" s="8" t="n">
+        <v>30</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:AH1"/>

</xml_diff>